<commit_message>
F1-A/B data-driven: enemies.scaling + waves.generation + routes.boss_wave 参数化接入
- T-001/002: enemies.json.scaling 公式字符串 → 参数（speed_growth_per_wave/cap/reduction + elite_hp/dmg_mult_per_wave），get_scaled_enemy 消费；删死公式列
- T-003: waves.json.generation → 参数（spawn_interval_min/decay）接入 enemy_spawner
- T-014: routes.json.boss_wave=10 接入 route_generator（generate_from + _reassign_wave_indices 读 DataLoader）
- 改 Excel enemy_scaling speed_reduction 0.5→0.4 实测生效（chaser w10 移速 176→140.8）
- day30_f1_scaling_check.gd 探针 10 断言（数值零漂移：chaser hp23/speed176、butcher w10 3000/14.4、predator 165、间隔 0.6、boss_wave 10）
- 回归套件 31 项/784 断言全绿；TECH_DEBT_ISSUES T-001/002/003/014 已收口、T-049 部分收口
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -1331,35 +1331,22 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>base_enemy_count_formula</t>
+          <t>spawn_interval_min</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>spawn_interval_formula</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>max_concurrent_formula</t>
-        </is>
-      </c>
+          <t>spawn_interval_decay</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>base_count + wave * 2</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>max(0.3, base_interval - wave * 0.02)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>min(20 + wave * 2, 60)</t>
-        </is>
+      <c r="A2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.02</v>
       </c>
     </row>
   </sheetData>
@@ -6106,7 +6093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6178,6 +6165,11 @@
           <t>constraints.max_battle_nodes</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>boss_wave</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -6214,6 +6206,9 @@
       </c>
       <c r="K2" t="n">
         <v>36</v>
+      </c>
+      <c r="L2" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -6248,7 +6243,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-10 00:56</t>
+          <t>- 生成时间：2026-08-10 01:04</t>
         </is>
       </c>
     </row>
@@ -18806,55 +18801,45 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>hp_formula</t>
+          <t>speed_growth_per_wave</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>damage_formula</t>
+          <t>speed_growth_cap</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>speed_formula</t>
+          <t>speed_reduction</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>elite_hp_multiplier</t>
+          <t>elite_hp_mult_per_wave</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>elite_damage_multiplier</t>
+          <t>elite_dmg_mult_per_wave</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>base_hp + hp_growth * wave</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>base_damage + damage_growth * wave</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>base_speed * (1 + min(wave * 0.01, 0.2)) * 0.5  # F-01(2026-08-06 用户拍板): 怪物移速降至50%</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1 + wave * 0.15</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1 + wave * 0.08</t>
-        </is>
+      <c r="A2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
F1-D T-010 shop params data-driven: reroll_cost(10)+core_grace_wave(4) -> stats.json shop 段(Excel stats_shop sheet 唯一事实源) + DataLoader.get_stats_shop() + shop.gd 读参兜底 + day30_f1d_shop_check 8 断言入 runner(31->32 项/792 断言) + 挂账 docs 收尾同步
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -28,7 +28,8 @@
     <sheet name="element_reactions" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="reaction_rules" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="routes" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="总览" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="stats_shop" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="总览" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -6220,6 +6221,40 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>reroll_cost</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>core_grace_wave</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -6243,7 +6278,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-10 01:04</t>
+          <t>- 生成时间：2026-08-10 08:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F1-G T-050 passive keys adjudication 22/22: 接线 5 键(xp_gain_percent->gain_exp / melee+ranged->分类伤害 / knockback->击退 / boss_elite_damage_percent->精英Boss增伤) + shop_weapon_upgrade 实为已消费(F31-3 服务池) + 13 键保留待F2+ + 3 键删数据登记(no_weapon_armor_bonus/special_enemies_next_wave/auto_turret_per_wave) + CONSUMED_BONUS_KEYS 白名单扩容 + excel_export 键注释/总览同步 + 回归 32/32(792) 全绿
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -6278,7 +6278,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-10 08:22</t>
+          <t>- 生成时间：2026-08-10 08:33</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6479,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>- 无消费方效果键 23 个（T-050，待 F1 逐键裁决）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, boss_elite_damage_percent, burn_duration_percent, damage_reduction_on_hit_percent, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, knockback, melee_damage, miss_chance_percent, no_weapon_armor_bonus, range, ranged_damage, reaction_heal, shop_weapon_upgrade, special_enemies_next_wave, structure_duration_percent, xp_gain_percent</t>
+          <t>- 无消费方效果键 17 个（T-050 已裁决：保留待 F2+/删数据）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, burn_duration_percent, damage_reduction_on_hit_percent, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, miss_chance_percent, no_weapon_armor_bonus, range, reaction_heal, special_enemies_next_wave, structure_duration_percent</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day30 F1-散 收口: 数值参数化散条目 8 项(T-007/008/009/011/012/013/015/053) - stats.combat/physics/skills三表+enemy_scaling冲锋3列, DataLoader三接口+兜底, 8消费点替换(含armor_cap无消费点登记T-054), 探针19/19双跑实证, 回归36/36 885断言, BASELINE CLEAN
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -29,7 +29,10 @@
     <sheet name="reaction_rules" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="routes" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="stats_shop" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="总览" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="stats_combat" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="stats_physics" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="stats_skills" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="总览" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -6898,6 +6901,260 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C0C0C0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>wave_clear_heal_ratio</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>max_waves</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>i_frames</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dodge_cap</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>debug_damage_mult</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>knockback_decay</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>contact_cooldown</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>armor_cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>通关回血比例</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>最大波次(兜底)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>受击无敌帧(秒)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>闪避上限</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>金手指受伤倍率</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>击退衰减(每帧)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>接触伤害冷却(秒)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>护甲减伤上限(保留参数)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C0C0C0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>projectile_mask</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>projectile_radius</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>弹丸碰撞层</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>弹丸碰撞半径</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C0C0C0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>fireball_speed</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>fireball_lifetime</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fireball_pierce</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>fireball_radius</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>火球速度</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>火球寿命(秒)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>火球穿透数</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>火球爆炸半径</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>280</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -6921,7 +7178,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-12 13:20</t>
+          <t>- 生成时间：2026-08-13 08:27</t>
         </is>
       </c>
     </row>
@@ -19729,7 +19986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19765,6 +20022,21 @@
           <t>elite_dmg_mult_per_wave</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>charge_speed_mult</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>charge_windup</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>charge_duration</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -19790,6 +20062,21 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>精英伤害每波倍率</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>冲锋倍率</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>蓄力间隔(秒)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>冲锋持续(秒)</t>
         </is>
       </c>
     </row>
@@ -19808,6 +20095,15 @@
       </c>
       <c r="E3" t="n">
         <v>0.08</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day30 BS-A 收口: 效果系统统一地基(A1~A5) - elements sheet升级effect表(数值零漂移, poison max_stacks=2) + StatusComponent通用组件(O1同源刷新/异源独立+max_stacks, dot/slow/stun/armor四类型) + apply_effect统一入口 + O2软控三类型运行时 + HUD玩家状态栏 + day30_effect 18/18; 回归39/39 936断言, BASELINE CLEAN
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -3273,7 +3273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3309,34 +3309,59 @@
           <t>effect</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>dot</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>dot_scaling</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>element_id</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>slow_percent</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>stun</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>armor_reduction</t>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>tick_interval</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>scaling_attr</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>scaling_ratio</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>target_attr</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>max_stacks</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>icon</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>vfx</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sfx</t>
         </is>
       </c>
     </row>
@@ -3363,32 +3388,57 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>持续伤害</t>
+          <t>元素ID</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>持续伤害成长</t>
+          <t>类型(dot/slow/stun/armor)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>元素ID</t>
+          <t>跳间隔(秒)</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>减速%</t>
+          <t>数值(跳伤/减速%/减防值)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>眩晕</t>
+          <t>缩放属性</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>护甲减伤</t>
+          <t>缩放比例</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>作用属性</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>叠加上限</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>图标</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>特效</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>音效</t>
         </is>
       </c>
     </row>
@@ -3411,16 +3461,37 @@
           <t>每秒造成 3 + (元素伤害×0.2) 点伤害</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" t="n">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>elemental_damage</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
         <v>0.2</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>fire</t>
-        </is>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -3442,14 +3513,33 @@
           <t>移动速度-40%</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>ice</t>
         </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>slow</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>40</v>
       </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>move_speed</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3470,12 +3560,31 @@
           <t>无法行动</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>lightning</t>
         </is>
       </c>
-      <c r="I5" t="b">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>stun</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3498,16 +3607,37 @@
           <t>每秒造成 2 + (元素伤害×0.15) 点伤害</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>poison</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>dot</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
         <v>2</v>
       </c>
-      <c r="F6" t="n">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>elemental_damage</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
         <v>0.15</v>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>poison</t>
-        </is>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -3529,13 +3659,32 @@
           <t>防御-5</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>plasma</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>defense</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -7178,7 +7327,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-13 08:27</t>
+          <t>- 生成时间：2026-08-13 09:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day30 BS-C 收口(C1~C4): boss_skill/boss_pattern表+enemies resist列(O5) + Boss pattern状态机(权重随机+保底不连续+phase 100/66/33解锁, 无pattern数据降级旧路径) + override合成 + day30_boss_skill 26/26(含§4); 回归40/40 962断言, BASELINE CLEAN
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -32,7 +32,9 @@
     <sheet name="stats_combat" sheetId="23" state="visible" r:id="rId23"/>
     <sheet name="stats_physics" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="stats_skills" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="总览" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="boss_skill" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="boss_pattern" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="总览" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -7304,6 +7306,392 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00E0B0B0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>telegraph</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>radius</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>arc</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>effects</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>resolve_delay</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>cooldown</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>vfx</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>warn_style</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>技能ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>预警时长(s)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>半径</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>扇形角(度,0=全圈)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>效果列表(JSON)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>结算延迟(s)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>直接伤害(结算时)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>冷却(s)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>特效</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>音效</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>预警样式</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>circle_aoe</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>circle</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>120</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>boss_skill</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>circle_eruption</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>circle</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>150</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>[{"source":"boss","id":"fire","duration":3,"dps":5}]</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H4" t="n">
+        <v>40</v>
+      </c>
+      <c r="I4" t="n">
+        <v>12</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>boss_skill</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00D0B0E0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>boss_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>skill_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>weight</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>override</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>min_interval</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BossID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>技能ID</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>随机权重</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>血量阶段(100/66/33)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>参数覆盖(JSON)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>最短释放间隔(s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>invoker</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>circle_aoe</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>invoker</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>circle_eruption</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>66</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"radius": 160}</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>predator</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>circle_aoe</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"damage": 25}</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -7327,7 +7715,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-13 09:31</t>
+          <t>- 生成时间：2026-08-13 09:42</t>
         </is>
       </c>
     </row>
@@ -18786,7 +19174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W25"/>
+  <dimension ref="A1:X25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18930,6 +19318,11 @@
           <t>phases</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>resist</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -19047,6 +19440,11 @@
           <t>阶段(JSON)</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>免疫列表(JSON, 硬控免疫软控保留)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -20082,6 +20480,11 @@
           <t>[{"hp_threshold_percent":100,"attacks":["summon_2_enemies_every_5s","3_projectile_spread"],"speed_multiplier":1.0},{"hp_threshold_percent":60,"attacks":["summon_4_enemies_every_2.5s","6_projectile_spread"],"speed_multiplier":1.2}]</t>
         </is>
       </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>["stun"]</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -20120,6 +20523,11 @@
       <c r="W25" t="inlineStr">
         <is>
           <t>[{"hp_threshold_percent":100,"attacks":["charge_attack","aoe_every_8s"],"speed_multiplier":1.0},{"hp_threshold_percent":66,"attacks":["charge_attack_2x","summon_1_elite","projectile_barrage"],"speed_multiplier":1.0},{"hp_threshold_percent":33,"attacks":["all_attacks_2x","summon_2_elite"],"speed_multiplier":1.3}]</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>["stun"]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PS-B(位移三型+invulnerable): boss_skill_factory扩展dash/blink/leap/spawn/buff(新增只加不改,既有4类型零触碰) + exec_dash/blink/leap/spawn/buff执行器(数据驱动三接口) + elements表新增invulnerable效果类型(Excel唯一事实源导出,0.3s默认) + status_component invulnerable置位/还原 + player.take_damage免疫窗口 + 合规白名单同步 + day31_skill_movement_check 13/13 + runner 48→49 + 回归49/49全绿BASELINE CLEAN
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -3275,7 +3275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3687,6 +3687,58 @@
       </c>
       <c r="L7" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>无敌</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Invulnerable</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>免疫伤害（位移技能窗口）</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>invulnerable</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>invulnerable</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>immune</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -7715,7 +7767,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-13 09:42</t>
+          <t>- 生成时间：2026-08-16 00:54</t>
         </is>
       </c>
     </row>
@@ -7879,7 +7931,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>## elements（5 行）</t>
+          <t>## elements（6 行）</t>
         </is>
       </c>
     </row>
@@ -15542,7 +15594,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -15569,6 +15621,9 @@
           <t>["damage"]</t>
         </is>
       </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -15608,7 +15663,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -15649,7 +15704,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -15676,6 +15731,9 @@
           <t>["range"]</t>
         </is>
       </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -15701,6 +15759,9 @@
           <t>["harvesting"]</t>
         </is>
       </c>
+      <c r="I9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -15740,7 +15801,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -15767,6 +15828,9 @@
           <t>["dodge"]</t>
         </is>
       </c>
+      <c r="I11" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -15792,6 +15856,9 @@
           <t>["elemental"]</t>
         </is>
       </c>
+      <c r="I12" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -15817,6 +15884,9 @@
           <t>["melee"]</t>
         </is>
       </c>
+      <c r="I13" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -15842,6 +15912,9 @@
           <t>["ranged"]</t>
         </is>
       </c>
+      <c r="I14" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15881,7 +15954,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
@@ -15922,7 +15995,7 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
@@ -15949,6 +16022,9 @@
           <t>["engineering"]</t>
         </is>
       </c>
+      <c r="I17" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15974,6 +16050,9 @@
           <t>["dodge"]</t>
         </is>
       </c>
+      <c r="I18" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15999,6 +16078,9 @@
           <t>["melee"]</t>
         </is>
       </c>
+      <c r="I19" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -16038,7 +16120,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
@@ -16079,7 +16161,7 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -16120,7 +16202,7 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23">
@@ -16147,6 +16229,9 @@
           <t>["elemental","hp_regen"]</t>
         </is>
       </c>
+      <c r="I23" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -16172,6 +16257,9 @@
           <t>["speed","engineering"]</t>
         </is>
       </c>
+      <c r="I24" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -16197,6 +16285,9 @@
           <t>["crit"]</t>
         </is>
       </c>
+      <c r="I25" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -16222,6 +16313,9 @@
           <t>["damage"]</t>
         </is>
       </c>
+      <c r="I26" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -16261,7 +16355,7 @@
         </is>
       </c>
       <c r="I27" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28">
@@ -16302,7 +16396,7 @@
         </is>
       </c>
       <c r="I28" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29">
@@ -16329,6 +16423,9 @@
           <t>["melee","attack_speed"]</t>
         </is>
       </c>
+      <c r="I29" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -16354,6 +16451,9 @@
           <t>["melee","ranged","engineering","crit","elemental"]</t>
         </is>
       </c>
+      <c r="I30" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -16393,7 +16493,7 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32">
@@ -16434,7 +16534,7 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33">
@@ -16461,6 +16561,9 @@
           <t>["damage"]</t>
         </is>
       </c>
+      <c r="I33" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -16486,6 +16589,9 @@
           <t>["damage"]</t>
         </is>
       </c>
+      <c r="I34" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -16525,7 +16631,7 @@
         </is>
       </c>
       <c r="I35" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36">
@@ -16566,7 +16672,7 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37">
@@ -16593,6 +16699,9 @@
           <t>["range"]</t>
         </is>
       </c>
+      <c r="I37" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -16618,6 +16727,9 @@
           <t>["elemental"]</t>
         </is>
       </c>
+      <c r="I38" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -16643,6 +16755,9 @@
           <t>["engineering"]</t>
         </is>
       </c>
+      <c r="I39" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -16668,6 +16783,9 @@
           <t>[]</t>
         </is>
       </c>
+      <c r="I40" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -16693,6 +16811,9 @@
           <t>["attack_speed","damage"]</t>
         </is>
       </c>
+      <c r="I41" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -16718,6 +16839,9 @@
           <t>["damage"]</t>
         </is>
       </c>
+      <c r="I42" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -16743,6 +16867,9 @@
           <t>["ranged"]</t>
         </is>
       </c>
+      <c r="I43" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -16768,6 +16895,9 @@
           <t>["damage"]</t>
         </is>
       </c>
+      <c r="I44" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -16807,7 +16937,7 @@
         </is>
       </c>
       <c r="I45" t="n">
-        <v>12</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46">
@@ -16834,6 +16964,9 @@
           <t>["elemental"]</t>
         </is>
       </c>
+      <c r="I46" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -16859,6 +16992,9 @@
           <t>["engineering"]</t>
         </is>
       </c>
+      <c r="I47" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -16898,7 +17034,7 @@
         </is>
       </c>
       <c r="I48" t="n">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="J48" t="b">
         <v>1</v>
@@ -16965,7 +17101,7 @@
         </is>
       </c>
       <c r="I49" t="n">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="J49" t="b">
         <v>1</v>
@@ -17032,7 +17168,7 @@
         </is>
       </c>
       <c r="I50" t="n">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="J50" t="b">
         <v>1</v>
@@ -17085,6 +17221,9 @@
           <t>["relic"]</t>
         </is>
       </c>
+      <c r="I51" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -17116,7 +17255,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>20</v>
+        <v>49</v>
       </c>
     </row>
     <row r="53">
@@ -17149,7 +17288,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>21</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54">
@@ -17190,7 +17329,7 @@
         </is>
       </c>
       <c r="I54" t="n">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="P54" t="inlineStr">
         <is>
@@ -17242,7 +17381,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="P55" t="inlineStr">
         <is>
@@ -17291,7 +17430,7 @@
         </is>
       </c>
       <c r="I56" t="n">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="P56" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
PS-C+E(skill_relics掉落+局外等级解锁): 新表skill_relics(3掉落,dash/blink/leap per_character变体)/skill_unlocks(局外门槛表Lv2/Lv4解锁槽1/2, Excel唯一事实源) + DataLoader接口(get_skill_relics_by_source/resolve_relic_skill/get_unlocked_slots_for_level) + enemy_damage掉落钩子(精英80%三选一/章Boss必掉+PS-E2解锁槽装配) + 剑士星刃→剑气爆发(se_skill_sword_arc扇形贯穿,day3探针同步) + SaveSystem skill_slots持久化(load_meta扩展键) + day31_skill_relic 9/9 + day31_skill_levelup 7/7 + runner 50→51 + 回归51/51全绿BASELINE CLEAN
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -34,7 +34,9 @@
     <sheet name="stats_skills" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="boss_skill" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="boss_pattern" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="总览" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="skill_relics" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="skill_unlocks" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="总览" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -7744,231 +7746,227 @@
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t># 数据分布总览（DATA_OVERVIEW）</t>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>base_type</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>drop_source</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>per_character</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>基础类型</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>掉落源</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>按角色变体(JSON)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-16 00:54</t>
+          <t>relic_dash</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>疾风冲刺</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>向前冲刺一段距离，期间无敌</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>dash</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>{"se_irene":{"type":"dash","params":{"distance":140,"cooldown":8}},"se_noa":{"type":"dash","params":{"distance":160,"cooldown":9}},"se_ren":{"type":"dash","params":{"distance":120,"cooldown":7}}}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>- 来源：docs/GameData.xlsx（tools/excel_export.py 导出时自动刷新）</t>
+          <t>relic_blink</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>相位闪现</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>瞬移到目标位置，可穿怪</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>blink</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>{"se_irene":{"type":"blink","params":{"distance":220,"cooldown":12}},"se_noa":{"type":"blink","params":{"distance":240,"cooldown":13}},"se_ren":{"type":"blink","params":{"distance":200,"cooldown":11}}}</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>## weapons（36 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>- 分类分布：{'melee': 9, 'ranged': 9, 'elemental': 10, 'engineering': 8}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>- 等级条目：288（36 把 × 8 级）</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>- 基础 damage：min 0.0 / max 45.0 / 均值 11.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>- 基础 cooldown：min 0.05 / max 2.0 / 均值 0.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>- 基础 range：min 100.0 / max 400.0 / 均值 214.4</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>## items（54 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>- 稀有度分布：{'common': 15, 'uncommon': 12, 'rare': 12, 'legendary': 13, 'epic': 2}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>- 效果键 Top（共 36 种）：damage_percent×14, max_hp×8, attack_speed_percent×7, armor×7, speed_percent×7, dodge_percent×6, elemental_damage×6, melee_damage×6</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>- price：min 0.0 / max 120.0 / 均值 57.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>## enemies（23 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>- 分类分布：{'regular': 15, 'elite': 6, 'boss': 2}</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>## characters（10 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>- 起始武器 10 把：pistol, fist, slingshot, wand, turret, dagger, se_star_flame, se_auto_turret, se_star_blade, se_holy_staff</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>## waves（20 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>- 波次范围：1 – 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>## events（10 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>## stats（20 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>## elements（6 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>## element_reactions（10 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>## routes（1 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>## 关注项</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>- 无消费方效果键 17 个（T-050 已裁决：保留待 F2+/删数据）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, burn_duration_percent, damage_reduction_on_hit_percent, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, miss_chance_percent, no_weapon_armor_bonus, range, reaction_heal, special_enemies_next_wave, structure_duration_percent</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>relic_leap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>破空跃击</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>跃向目标点，落地范围伤害</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>leap</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>chapter_boss</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>{"se_irene":{"type":"leap","params":{"distance":170,"land_radius":70,"damage":45,"cooldown":10}},"se_noa":{"type":"leap","params":{"distance":190,"land_radius":80,"damage":40,"cooldown":11}},"se_ren":{"type":"leap","params":{"distance":150,"land_radius":60,"damage":55,"cooldown":9}}}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>char_level</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>unlocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>角色等级</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>解锁内容(JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"slot":1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"slot":2}</t>
         </is>
       </c>
     </row>
@@ -15254,6 +15252,242 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00808080"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t># 数据分布总览（DATA_OVERVIEW）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>- 生成时间：2026-08-16 01:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>- 来源：docs/GameData.xlsx（tools/excel_export.py 导出时自动刷新）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>## weapons（36 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>- 分类分布：{'melee': 9, 'ranged': 9, 'elemental': 10, 'engineering': 8}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>- 等级条目：288（36 把 × 8 级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>- 基础 damage：min 0.0 / max 45.0 / 均值 11.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>- 基础 cooldown：min 0.05 / max 2.0 / 均值 0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>- 基础 range：min 100.0 / max 400.0 / 均值 214.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>## items（54 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- 稀有度分布：{'common': 15, 'uncommon': 12, 'rare': 12, 'legendary': 13, 'epic': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- 效果键 Top（共 36 种）：damage_percent×14, max_hp×8, attack_speed_percent×7, armor×7, speed_percent×7, dodge_percent×6, elemental_damage×6, melee_damage×6</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>- price：min 0.0 / max 120.0 / 均值 57.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>## enemies（23 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>- 分类分布：{'regular': 15, 'elite': 6, 'boss': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>## characters（10 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>- 起始武器 10 把：pistol, fist, slingshot, wand, turret, dagger, se_star_flame, se_auto_turret, se_star_blade, se_holy_staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>## waves（20 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>- 波次范围：1 – 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>## events（10 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>## stats（20 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>## elements（6 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>## element_reactions（10 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>## routes（1 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>## 关注项</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>- 无消费方效果键 17 个（T-050 已裁决：保留待 F2+/删数据）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, burn_duration_percent, damage_reduction_on_hit_percent, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, miss_chance_percent, no_weapon_armor_bonus, range, reaction_heal, special_enemies_next_wave, structure_duration_percent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21840,30 +22074,36 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>se_skill_blade_burst</t>
+          <t>se_skill_sword_arc</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>星刃爆发</t>
+          <t>剑气爆发</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Blade Burst</t>
+          <t>Sword Arc</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>arc</t>
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="R11" t="n">
+        <v>25</v>
+      </c>
+      <c r="S11" t="n">
+        <v>120</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>5 秒内环绕星刃额外 +3 把并提升 50% 攻速</t>
+          <t>向前挥出扇形剑气，贯穿敌人一次爆发</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -21875,15 +22115,6 @@
         <is>
           <t>暴击吸血成长：每级 +1% 暴击率 / +0.5% 生命偷取</t>
         </is>
-      </c>
-      <c r="AC11" t="n">
-        <v>5</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>3</v>
-      </c>
-      <c r="AG11" t="n">
-        <v>50</v>
       </c>
       <c r="AH11" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
PS-D(章节化数据层+阻塞登记): routes.json chapters字段落地(4章定义3/4/4/4+章末类型章1=event章2-4=boss, Excel唯一事实源) + day31_chapter_check 5/5 + boss_layers映射调整执行阻塞(F-27用户拍板双Boss[9,14] vs 章2/3/4三Boss[7,11,15]冲突,按方案R5兜底回滚交方案师裁决) + SOLUTION_PLAN执行结果 + runner 51→52 + 回归52/52全绿BASELINE CLEAN
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -6871,7 +6871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6948,6 +6948,11 @@
           <t>boss_wave</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>chapters</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7008,6 +7013,11 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>Boss波次</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>章节定义(JSON: chapter_id/layers/end_type)</t>
         </is>
       </c>
     </row>
@@ -7049,6 +7059,11 @@
       </c>
       <c r="L3" t="n">
         <v>10</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>[{"chapter_id":1,"layers":[1,2,3],"end_type":"event"},{"chapter_id":2,"layers":[4,5,6,7],"end_type":"boss"},{"chapter_id":3,"layers":[8,9,10,11],"end_type":"boss"},{"chapter_id":4,"layers":[12,13,14,15],"end_type":"boss"}]</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -15282,7 +15297,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-16 01:01</t>
+          <t>- 生成时间：2026-08-16 01:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31 总指挥第4轮: F1-E第一批enemy精灵表现抽表(Excel enemy_sprites sheet 23敌+presentation.json+DataLoader消费246断言探针) + AUDIO_FEEL O-1~3拍板(M1+M2/近重远轻/H1挂P2) + HUD se_skill_sword_arc图标映射探针22断言 + TASKS/SOLUTION_PLAN/COMMAND_LOG台账
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -14,29 +14,30 @@
     <sheet name="items_effects" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="enemies" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="enemy_scaling" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="characters" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="characters_passives" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="characters_penalties" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="waves" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="wave_generation" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="wave_rewards" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="events" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="stats" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="stats_formulas" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="stats_leveling" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="elements" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="element_reactions" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="reaction_rules" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="routes" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="stats_shop" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="stats_combat" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="stats_physics" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="stats_skills" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="boss_skill" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="boss_pattern" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="skill_relics" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="skill_unlocks" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="总览" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="enemy_sprites" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="characters" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="characters_passives" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="characters_penalties" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="waves" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="wave_generation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="wave_rewards" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="events" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="stats" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="stats_formulas" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="stats_leveling" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="elements" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="element_reactions" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="reaction_rules" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="routes" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="stats_shop" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="stats_combat" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="stats_physics" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="stats_skills" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="boss_skill" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="boss_pattern" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="skill_relics" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="skill_unlocks" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="总览" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -45,20 +46,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'items_effects'!$A$1:$C$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'enemies'!$A$1:$W$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'enemy_scaling'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'characters'!$A$1:$AM$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'characters_passives'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'characters_penalties'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'waves'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'wave_generation'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'wave_rewards'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'events'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'stats'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'stats_formulas'!$A$1:$O$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'stats_leveling'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'elements'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'element_reactions'!$A$1:$J$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'reaction_rules'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'routes'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'characters'!$A$1:$AM$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'characters_passives'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'characters_penalties'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'waves'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'wave_generation'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'wave_rewards'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'events'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'stats'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'stats_formulas'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'stats_leveling'!$A$1:$C$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'elements'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'element_reactions'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'reaction_rules'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'routes'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -580,6 +581,510 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>char_id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>角色ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>效果键</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>well_rounded</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>max_hp</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>well_rounded</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>speed_percent</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>well_rounded</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>harvesting</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>brawler</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>melee_attack_speed_percent</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>brawler</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>melee_damage</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>brawler</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>life_steal_percent</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ranger</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ranged_range_bonus</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ranger</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ranged_damage_effect_percent</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ranger</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>crit_chance_percent</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>elemental_damage</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>double_element_chance_percent</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>mage</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>elemental_damage_effect_percent</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>engineering</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>structure_hp_percent</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>engineer</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>structure_damage_percent</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>gambler</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>gambler</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>shop_quality_percent</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>gambler</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>double_material_chance_percent</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>se_irene</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>elemental_damage</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>se_irene</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>fire_damage_percent</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>se_irene</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>burn_duration_percent</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>se_noa</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>engineering</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>se_noa</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>structure_hp_percent</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>se_noa</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>summon_count</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>se_ren</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>melee_damage</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>se_ren</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>crit_chance_percent</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>se_ren</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>life_steal_percent</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>se_siia</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>hp_regen</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>se_siia</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>max_hp</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>se_siia</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -883,7 +1388,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1375,7 +1880,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1428,7 +1933,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1498,7 +2003,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2253,7 +2758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2943,7 +3448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3206,7 +3711,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3275,7 +3780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3745,462 +4250,6 @@
         <is>
           <t>1</t>
         </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:J1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>combination</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>name_en</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>damage</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>damage_scaling</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>aoe_radius</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>extra_effect</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>chain_count</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>chain_falloff</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>组合(JSON)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>名称</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>英文名</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>伤害</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>伤害成长</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>范围半径</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>附加效果</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>序号</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>连锁数</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>连锁衰减</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>["fire","ice"]</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>蒸汽爆破</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Steam Burst</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>80</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>致盲(命中率-50%) 2秒</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>["fire","lightning"]</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>雷火风暴</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Storm of Fire</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>触发3次连锁闪电</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="n">
-        <v>3</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>["fire","poison"]</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>瘟疫之火</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Plague Fire</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>25</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>留下一片毒火区域(3秒, 每秒5点伤害)</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>["fire","plasma"]</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>超新星</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Supernova</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>40</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F6" t="n">
-        <v>120</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>无视护甲</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>["ice","lightning"]</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>超导</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Superconduct</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>冻结2秒</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>["ice","poison"]</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>寒毒</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Frost Toxin</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>8</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>减速延长至4秒且减速60%</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>["ice","plasma"]</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>绝对零度</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Absolute Zero</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>15</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>冻结3秒</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>["lightning","poison"]</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>腐蚀链</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Corrosive Chain</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>12</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>连锁敌人并施加中毒</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>8</v>
-      </c>
-      <c r="I10" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>["lightning","plasma"]</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>电磁脉冲</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>EMP</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>18</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>沉默敌人3秒(无法使用特殊技能)</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>["poison","plasma"]</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>衰变</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Decay</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>30</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>最大生命值-10% 持续整局</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -6781,6 +6830,462 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>combination</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>name_en</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>damage_scaling</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>aoe_radius</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>extra_effect</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>chain_count</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>chain_falloff</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>组合(JSON)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>伤害</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>伤害成长</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>范围半径</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>附加效果</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>连锁数</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>连锁衰减</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>["fire","ice"]</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>蒸汽爆破</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Steam Burst</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>80</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>致盲(命中率-50%) 2秒</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>["fire","lightning"]</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>雷火风暴</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Storm of Fire</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>触发3次连锁闪电</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>["fire","poison"]</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>瘟疫之火</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Plague Fire</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>留下一片毒火区域(3秒, 每秒5点伤害)</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>["fire","plasma"]</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>超新星</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Supernova</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>120</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>无视护甲</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>["ice","lightning"]</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>超导</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Superconduct</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>冻结2秒</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>["ice","poison"]</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>寒毒</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Frost Toxin</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>减速延长至4秒且减速60%</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>["ice","plasma"]</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>绝对零度</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Absolute Zero</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>冻结3秒</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>["lightning","poison"]</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>腐蚀链</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Corrosive Chain</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>连锁敌人并施加中毒</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>["lightning","plasma"]</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>电磁脉冲</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>EMP</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>18</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>沉默敌人3秒(无法使用特殊技能)</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>["poison","plasma"]</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>衰变</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Decay</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>30</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>最大生命值-10% 持续整局</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6862,7 +7367,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7069,7 +7574,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7115,7 +7620,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C0C0C0"/>
@@ -7243,7 +7748,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C0C0C0"/>
@@ -7293,7 +7798,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C0C0C0"/>
@@ -7369,7 +7874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E0B0B0"/>
@@ -7598,7 +8103,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00D0B0E0"/>
@@ -7755,7 +8260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7921,64 +8426,6 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>{"se_irene":{"type":"leap","params":{"distance":170,"land_radius":70,"damage":45,"cooldown":10}},"se_noa":{"type":"leap","params":{"distance":190,"land_radius":80,"damage":40,"cooldown":11}},"se_ren":{"type":"leap","params":{"distance":150,"land_radius":60,"damage":55,"cooldown":9}}}</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>char_level</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>unlocks</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>角色等级</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>解锁内容(JSON)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{"slot":1}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{"slot":2}</t>
         </is>
       </c>
     </row>
@@ -15252,6 +15699,64 @@
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>char_level</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>unlocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>角色等级</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>解锁内容(JSON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"slot":1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"slot":2}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -15275,7 +15780,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-18 03:24</t>
+          <t>- 生成时间：2026-08-18 05:02</t>
         </is>
       </c>
     </row>
@@ -21036,6 +21541,1117 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>size_w</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>size_h</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>move_frames</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>death_frames</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>move_fps</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>death_fps</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>hit_radius</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>tint</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>敌人ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>移动精灵</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>死亡精灵</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>精灵宽(px)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>精灵高(px)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>移动帧数</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>死亡帧数</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>移动FPS</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>死亡FPS</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>接触判定半径</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>色调(JSON)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>体型倍率</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>chaser</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>48</v>
+      </c>
+      <c r="E3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8</v>
+      </c>
+      <c r="J3" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>charger</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>48</v>
+      </c>
+      <c r="E4" t="n">
+        <v>48</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" t="n">
+        <v>8</v>
+      </c>
+      <c r="J4" t="n">
+        <v>28</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>[0.75, 0.85, 1.35]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>fly</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>48</v>
+      </c>
+      <c r="E5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="n">
+        <v>8</v>
+      </c>
+      <c r="I5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" t="n">
+        <v>28</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>[1.4, 1.2, 0.65]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>bruiser</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>48</v>
+      </c>
+      <c r="E6" t="n">
+        <v>48</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J6" t="n">
+        <v>28</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>[1.2, 0.9, 0.65]</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>spitter</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>48</v>
+      </c>
+      <c r="E7" t="n">
+        <v>48</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" t="n">
+        <v>6</v>
+      </c>
+      <c r="I7" t="n">
+        <v>8</v>
+      </c>
+      <c r="J7" t="n">
+        <v>28</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>[0.8, 1.1, 1.1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>healer</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>48</v>
+      </c>
+      <c r="E8" t="n">
+        <v>48</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>8</v>
+      </c>
+      <c r="J8" t="n">
+        <v>28</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>[1.15, 1.25, 1.05]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>spawner</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>48</v>
+      </c>
+      <c r="E9" t="n">
+        <v>48</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" t="n">
+        <v>8</v>
+      </c>
+      <c r="J9" t="n">
+        <v>28</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>[1.25, 0.8, 1.35]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>horned_charger</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_move.png</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_death.png</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>48</v>
+      </c>
+      <c r="E10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4</v>
+      </c>
+      <c r="H10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" t="n">
+        <v>8</v>
+      </c>
+      <c r="J10" t="n">
+        <v>28</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>[1.35, 0.8, 0.8]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>pursuer</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>48</v>
+      </c>
+      <c r="E11" t="n">
+        <v>48</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="n">
+        <v>8</v>
+      </c>
+      <c r="J11" t="n">
+        <v>28</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[1.35, 0.7, 1.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>slasher</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_move.png</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_death.png</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>48</v>
+      </c>
+      <c r="E12" t="n">
+        <v>48</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>6</v>
+      </c>
+      <c r="I12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J12" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>helmet_alien</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_move.png</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_death.png</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>48</v>
+      </c>
+      <c r="E13" t="n">
+        <v>48</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" t="n">
+        <v>8</v>
+      </c>
+      <c r="J13" t="n">
+        <v>28</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>[0.7, 1.0, 0.8]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>horned_fly</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_move.png</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_death.png</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>48</v>
+      </c>
+      <c r="E14" t="n">
+        <v>48</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I14" t="n">
+        <v>8</v>
+      </c>
+      <c r="J14" t="n">
+        <v>28</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>[1.35, 1.15, 0.6]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>corrupted_tree</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>48</v>
+      </c>
+      <c r="E15" t="n">
+        <v>48</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>8</v>
+      </c>
+      <c r="J15" t="n">
+        <v>28</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>[0.55, 0.85, 0.5]</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>mad_slasher</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_move.png</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/skeleton_death.png</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>48</v>
+      </c>
+      <c r="E16" t="n">
+        <v>48</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8</v>
+      </c>
+      <c r="I16" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" t="n">
+        <v>28</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>[1.4, 0.75, 0.75]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>lamprey</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_move.png</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/slime_death.png</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>48</v>
+      </c>
+      <c r="E17" t="n">
+        <v>48</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4</v>
+      </c>
+      <c r="H17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J17" t="n">
+        <v>28</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>[0.7, 0.8, 1.2]</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>butcher</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_move.png</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_death.png</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>64</v>
+      </c>
+      <c r="E18" t="n">
+        <v>64</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" t="n">
+        <v>8</v>
+      </c>
+      <c r="J18" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>colossus</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_move.png</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_death.png</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>64</v>
+      </c>
+      <c r="E19" t="n">
+        <v>64</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
+      <c r="I19" t="n">
+        <v>8</v>
+      </c>
+      <c r="J19" t="n">
+        <v>36</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>[1.2, 1.05, 0.8]</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>rhino</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_move.png</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_death.png</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>64</v>
+      </c>
+      <c r="E20" t="n">
+        <v>64</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" t="n">
+        <v>6</v>
+      </c>
+      <c r="I20" t="n">
+        <v>8</v>
+      </c>
+      <c r="J20" t="n">
+        <v>36</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>[1.1, 0.85, 0.9]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>monk</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_move.png</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_death.png</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>64</v>
+      </c>
+      <c r="E21" t="n">
+        <v>64</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" t="n">
+        <v>6</v>
+      </c>
+      <c r="I21" t="n">
+        <v>8</v>
+      </c>
+      <c r="J21" t="n">
+        <v>36</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>[0.85, 1.05, 0.9]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>croc</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_move.png</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_death.png</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>64</v>
+      </c>
+      <c r="E22" t="n">
+        <v>64</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" t="n">
+        <v>7</v>
+      </c>
+      <c r="I22" t="n">
+        <v>8</v>
+      </c>
+      <c r="J22" t="n">
+        <v>36</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>[0.9, 1.15, 0.75]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>mom</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_move.png</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/elite_death.png</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>64</v>
+      </c>
+      <c r="E23" t="n">
+        <v>64</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" t="n">
+        <v>5</v>
+      </c>
+      <c r="I23" t="n">
+        <v>8</v>
+      </c>
+      <c r="J23" t="n">
+        <v>36</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>[1.1, 0.8, 1.1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>invoker</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/invoker_move.png</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/invoker_death.png</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>128</v>
+      </c>
+      <c r="E24" t="n">
+        <v>128</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" t="n">
+        <v>8</v>
+      </c>
+      <c r="J24" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>predator</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/predator_move.png</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/enemies/predator_death.png</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>128</v>
+      </c>
+      <c r="E25" t="n">
+        <v>128</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>6</v>
+      </c>
+      <c r="I25" t="n">
+        <v>8</v>
+      </c>
+      <c r="J25" t="n">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -22231,508 +23847,4 @@
   <autoFilter ref="A1:AM1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>char_id</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>key</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>角色ID</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>效果键</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>数值</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>well_rounded</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>max_hp</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>well_rounded</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>speed_percent</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>well_rounded</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>harvesting</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>brawler</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>melee_attack_speed_percent</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>brawler</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>melee_damage</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>brawler</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>life_steal_percent</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ranger</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>ranged_range_bonus</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ranger</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ranged_damage_effect_percent</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ranger</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>crit_chance_percent</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>mage</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>elemental_damage</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>mage</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>double_element_chance_percent</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>mage</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>elemental_damage_effect_percent</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>engineer</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>engineer</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>structure_hp_percent</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>engineer</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>structure_damage_percent</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>gambler</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>gambler</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>shop_quality_percent</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>gambler</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>double_material_chance_percent</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>se_irene</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>elemental_damage</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>se_irene</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>fire_damage_percent</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>se_irene</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>burn_duration_percent</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>se_noa</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>engineering</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>se_noa</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>structure_hp_percent</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>se_noa</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>summon_count</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>se_ren</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>melee_damage</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>se_ren</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>crit_chance_percent</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>se_ren</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>life_steal_percent</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>se_siia</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>hp_regen</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>se_siia</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>max_hp</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>se_siia</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:C1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Day31 执行者第56轮: F1-E第二批BEHAVIOR_MAP抽表闭环——Excel enemy_behavior表(9行)+data_schema注册+excel_export构建+presentation.json behavior_map 9条(13 JSON零diff)+data_loader get_enemy_behavior(懒加载+枚举名解析+const兜底)+enemy.gd行为解析改读+探针261/261+回归60/60
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -37,7 +37,8 @@
     <sheet name="boss_pattern" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="skill_relics" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="skill_unlocks" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="总览" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="enemy_behavior" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="总览" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -15757,6 +15758,156 @@
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>behavior</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>行为字符串</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>行为枚举</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>chase</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CHASE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>charge</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CHARGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>zigzag</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ZIGZAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ranged</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>RANGED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HEAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>spawn</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SPAWN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>stationary</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>STATIONARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>aoe_attack</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AOE_ATTACK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>self_heal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SELF_HEAL</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -15780,7 +15931,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-18 05:02</t>
+          <t>- 生成时间：2026-08-18 05:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31 执行者第57轮: AUDIO_FEEL AF-P0 批A-C全收口——hitstop顿帧系统(新hitstop_controller trigger取max+create_timer ignore_time_scale恢复+超时兜底, projectile/melee_sweep/enemy_damage接线, O-2近重0.15远轻0.05) + 相机震屏分级(light/medium/heavy表化零漂移+_trigger_camera_shake+3调用点) + 音画同步(play_sfx_delayed+暴击crit音, death/skill核对防双播) + Excel stats_feel段10键(其余13 JSON零diff)+get_stats_feel兜底 + day31_feel_check 26/26 + 回归61/61(1489断言)+BASELINE CLEAN + PLAYTEST AF-P0主观回归面
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -38,7 +38,8 @@
     <sheet name="skill_relics" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="skill_unlocks" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="enemy_behavior" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="总览" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="stats_feel" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="总览" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -15908,6 +15909,156 @@
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>hitstop_melee</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hitstop_ranged</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>hitstop_crit_bonus</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>hitstop_boss_kill</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>shake_light_duration</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>shake_light_magnitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>shake_medium_duration</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>shake_medium_magnitude</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>shake_heavy_duration</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>shake_heavy_magnitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>顿帧-近战(秒)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>顿帧-远程(秒)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>顿帧-暴击追加(秒)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>顿帧-Boss击杀(秒)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>震屏-轻-时长(秒)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>震屏-轻-幅度</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>震屏-中-时长(秒)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>震屏-中-幅度</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>震屏-重-时长(秒)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>震屏-重-幅度</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -15931,7 +16082,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-18 05:28</t>
+          <t>- 生成时间：2026-08-18 07:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31-F1-E3-BGM/SFX抽表收口(总指挥第5轮): audio_config sheet 12行(id/category/path) + data_schema注册 + excel_export audio_map构建 + 导出12键零漂移(其余13 JSON零diff) + DataLoader.get_audio_config懒加载 + audio_manager._resolve_audio_path消费改读(BGM_MAP/SFX_MAP const保留兜底, 红线2键契约零破坏) + day31_presentation_check +§3 audio段12断言→273/273 + day24_audio_check 14/14零改动 + 端到端双跑PASS + 全量回归61/61(1504断言) + baseline CLEAN + TASKS F1-E行3/7批 + TECH_DEBT_ISSUES T-016/017/018转已收口
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -38,8 +38,9 @@
     <sheet name="skill_relics" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="skill_unlocks" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="enemy_behavior" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="stats_feel" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="总览" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="audio_config" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="stats_feel" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="总览" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$1</definedName>
@@ -15912,143 +15913,250 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>hitstop_melee</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>hitstop_ranged</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>hitstop_crit_bonus</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>hitstop_boss_kill</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>shake_light_duration</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>shake_light_magnitude</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>shake_medium_duration</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>shake_medium_magnitude</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>shake_heavy_duration</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>shake_heavy_magnitude</t>
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>path</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>顿帧-近战(秒)</t>
+          <t>音频ID</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>顿帧-远程(秒)</t>
+          <t>类别(bgm/sfx)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>顿帧-暴击追加(秒)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>顿帧-Boss击杀(秒)</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>震屏-轻-时长(秒)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>震屏-轻-幅度</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>震屏-中-时长(秒)</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>震屏-中-幅度</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>震屏-重-时长(秒)</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>震屏-重-幅度</t>
+          <t>资源路径</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="B3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="H3" t="n">
-        <v>6</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J3" t="n">
-        <v>9</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>menu</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bgm</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>res://assets/audio/bgm/bgm_menu.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>battle</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>bgm</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>res://assets/audio/bgm/bgm_battle.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/hit.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>crit</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/crit.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/death.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>levelup</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/levelup.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>coin</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/coin.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>shop</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/shop.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/skill.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/heal.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/event.wav</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>boss</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>res://assets/audio/sfx/boss.wav</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -16057,6 +16165,156 @@
 </file>
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>hitstop_melee</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>hitstop_ranged</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>hitstop_crit_bonus</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>hitstop_boss_kill</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>shake_light_duration</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>shake_light_magnitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>shake_medium_duration</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>shake_medium_magnitude</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>shake_heavy_duration</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>shake_heavy_magnitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>顿帧-近战(秒)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>顿帧-远程(秒)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>顿帧-暴击追加(秒)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>顿帧-Boss击杀(秒)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>震屏-轻-时长(秒)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>震屏-轻-幅度</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>震屏-中-时长(秒)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>震屏-中-幅度</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>震屏-重-时长(秒)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>震屏-重-幅度</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00808080"/>
@@ -16082,7 +16340,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-18 07:36</t>
+          <t>- 生成时间：2026-08-18 19:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F-45 手感三连修复(用户08-18直派): 顿帧四档调小0.15/0.05/0.1/0.15->0.03/0.02/0.02/0.06(Excel stats_feel数据驱动, 低频1-2击/s无感、1s5击+高频才见节奏顿挫) + 震屏条件收紧(普攻命中零震屏, projectile仅se_skill技能弹丸震/melee_sweep删命中震屏; 击杀medium/heavy+玩家受伤light保留) + hit命中特效手感覆盖(scale0.6调小+alpha0.55半透明+播完0.25s渐隐不突然消失, FX_FEEL_OVERRIDE独立配置FX_CONFIG 10键零改动) + day31_feel_check断言同步, 护栏feel26/26+vfx18/18+attack20/20+presentation273/273+flee18/18+boss_after6/6+fb5 29/29+全量回归62/62 1534断言全绿
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -16279,16 +16279,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.15</v>
+        <v>0.03</v>
       </c>
       <c r="B3" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="D3" t="n">
-        <v>0.15</v>
+        <v>0.06</v>
       </c>
       <c r="E3" t="n">
         <v>0.15</v>
@@ -16340,7 +16340,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-18 21:16</t>
+          <t>- 生成时间：2026-08-18 21:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31-F1-E-4-1 FX抽表数据侧收口(总指挥第6轮): GameData.xlsx新增fx_config sheet(10行×id/frames/fps/path/size_w/size_h, 值逐一抄自vfx_player.gd FX_CONFIG) + data_schema注册fx_config(presentation.json/fx_config/dict/id) + excel_export presentation段追加fx_map构建(size_w/size_h->{"x","y"}组装) + 导出fx_config 10键零漂移(其余14 JSON零diff) — 用户08-18 23:1x拍板#3直接执行决策落地前已动工, 提交为检查点交接#3续做4-2~EXIT
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -39,7 +39,8 @@
     <sheet name="enemy_behavior" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="audio_config" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="stats_feel" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="总览" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="fx_config" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="总览" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$38</definedName>
@@ -70,7 +71,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -256,6 +257,9 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="35">
@@ -718,13 +722,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -16940,6 +16945,324 @@
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>frames</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>fps</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>size_w</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>size_h</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>特效ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>帧数</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>帧率(fps)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>资源路径</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>尺寸宽</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>尺寸高</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_hit.png</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F3" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>crit</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_crit.png</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>32</v>
+      </c>
+      <c r="F4" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_death.png</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F5" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>levelup</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_levelup.png</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>32</v>
+      </c>
+      <c r="F6" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pickup</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_pickup.png</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fireball</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_fireball.png</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>64</v>
+      </c>
+      <c r="F8" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>turret_deploy</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_turret_deploy.png</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>64</v>
+      </c>
+      <c r="F9" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>blade_burst</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_blade_burst.png</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>64</v>
+      </c>
+      <c r="F10" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>meteor</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" t="n">
+        <v>12</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_meteor.png</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>128</v>
+      </c>
+      <c r="F11" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/effects/fx_shield.png</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>64</v>
+      </c>
+      <c r="F12" t="n">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -16963,7 +17286,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-18 22:40</t>
+          <t>- 生成时间：2026-08-18 23:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31-LD-A1~A3+EXIT LEVEL_DESIGN数据地基: spawn_points/boss_phase_events两新sheet(11点位三型/7事件6类型) + waves加spawn_set/spawn_order列(1/10/20波示例) + data_schema注册 + excel_export构建分组排序+FK校验三态+顺手修--check-only只读缺陷 + DataLoader三接口(get_spawn_points/get_spawn_set/get_boss_phase_events懒加载) + day31_level_design_data_check 24/24 + runner 63->64件套/day26 1578->1602锚点同步
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -40,7 +40,9 @@
     <sheet name="audio_config" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="stats_feel" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="fx_config" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="总览" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="spawn_points" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="boss_phase_events" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="总览" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$38</definedName>
@@ -262,7 +264,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -465,6 +467,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -722,7 +730,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -730,6 +738,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2040,7 +2049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2049,6 +2058,8 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2082,6 +2093,16 @@
           <t>special_note</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>spawn_set</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>spawn_order</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2112,6 +2133,16 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>特殊备注</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>出生点组(JSON数组)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>点位轮换(sequence/random)</t>
         </is>
       </c>
     </row>
@@ -2130,6 +2161,16 @@
           <t>[{"enemy":"chaser","count":8},{"enemy":"fly","count":4}]</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>["north","east","ring_outer"]</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>sequence</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2314,6 +2355,16 @@
           <t>Boss持续生成普通敌人</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>["boss_top"]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>sequence</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2517,6 +2568,16 @@
       <c r="F22" t="inlineStr">
         <is>
           <t>最终Boss持续生成精英和普通敌人</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>["arena_center"]</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>sequence</t>
         </is>
       </c>
     </row>
@@ -17263,6 +17324,628 @@
 <file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>point_id</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>direction</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>radius</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>inset</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>min_dist_player</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>点位ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>类型(edge/anchor/ring)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>方位(n/s/e/w/ne/nw/se/sw)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>锚点X(0~1比例)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>锚点Y(0~1比例)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>半径(px)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>边缘内缩(px)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>离玩家最小距离(px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H3" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>40</v>
+      </c>
+      <c r="H4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>east</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>east</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>west</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>west</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>40</v>
+      </c>
+      <c r="H7" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>nw</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>nw</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>40</v>
+      </c>
+      <c r="H8" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>se</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>se</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>40</v>
+      </c>
+      <c r="H9" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>sw</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>40</v>
+      </c>
+      <c r="H10" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>boss_top</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>edge</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>60</v>
+      </c>
+      <c r="H11" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>arena_center</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>anchor</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H12" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ring_outer</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>300</v>
+      </c>
+      <c r="H13" t="n">
+        <v>110</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>boss_id</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>hp_threshold_percent</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>seq</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>event_type</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>param</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>once</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BossID(FK→enemies)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>血线阈值%(1~99,100=开局登场)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>同阈值顺序(1起)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>类型(banner/vfx/sfx/dialogue/camera/buff)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>参数(JSON)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>只触发一次(1/0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>invoker</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"text":"炼金暴君 现身！","color":"#E24B4A","duration":1.5}</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>invoker</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>60</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"text":"狂怒！火力全开","color":"#E24B4A","duration":1.5}</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>invoker</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>buff</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"target":"self","effect":"frenzy","duration":10}</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>invoker</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>40</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>camera</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"strength":"heavy","count":2}</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>predator</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>dialogue</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"text":"猎杀开始……","speaker":"predator"}</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>predator</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>66</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>vfx</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"name":"blade_burst"}</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>predator</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>33</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>sfx</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"name":"boss"}</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -17286,7 +17969,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-19 00:41</t>
+          <t>- 生成时间：2026-08-19 02:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31-F1-E-6-1 T-004 初始枪抽表数据侧(#3): weapons sheet +starting_gun行(8/0.4/180/knockback0/max1 ranged归组, price/crit/icon/special留空=JSON键缺失=build兜底默认与内联Weapon.new一致, projectile_speed/lifetime不进表, levels空) + excel_export导出 ranged10把 其余16JSON零diff
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -4963,7 +4963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH38"/>
+  <dimension ref="A1:AH39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="2"/>
@@ -7513,6 +7513,46 @@
         <v>3</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>starting_gun</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>初始枪</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Starting Gun</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>8</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H39" t="n">
+        <v>180</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>ranged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AG38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17969,7 +18009,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-19 02:40</t>
+          <t>- 生成时间：2026-08-19 06:40</t>
         </is>
       </c>
     </row>
@@ -17986,14 +18026,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>## weapons（36 行）</t>
+          <t>## weapons（37 行）</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>- 分类分布：{'melee': 9, 'ranged': 9, 'elemental': 10, 'engineering': 8}</t>
+          <t>- 分类分布：{'melee': 9, 'ranged': 10, 'elemental': 10, 'engineering': 8}</t>
         </is>
       </c>
     </row>
@@ -18007,7 +18047,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- 基础 damage：min 0.0 / max 45.0 / 均值 11.9</t>
+          <t>- 基础 damage：min 0.0 / max 45.0 / 均值 11.8</t>
         </is>
       </c>
     </row>
@@ -18021,7 +18061,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- 基础 range：min 100.0 / max 400.0 / 均值 214.4</t>
+          <t>- 基础 range：min 100.0 / max 400.0 / 均值 213.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31-F1-E-6-3 T-022 skill_icon_map抽表数据侧(#3): 新增skill_icon_map sheet 5行(id/icon_index双行表头 与SKILL_ICON_MAP const现值0-4逐一一致) + data_schema注册(dict形id主键 仿fx_config) + excel_export presentation段追加解析(id->int(icon_index)) + files dict第6键 其余16JSON零diff
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -42,7 +42,8 @@
     <sheet name="fx_config" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="spawn_points" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="boss_phase_events" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="总览" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="skill_icon_map" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="总览" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$38</definedName>
@@ -17986,6 +17987,94 @@
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>icon_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>技能ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>图标帧索引</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>se_skill_fireball</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>se_skill_deploy_turret</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>se_skill_blade_burst</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>se_skill_holy_shield</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>se_skill_sword_arc</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -18009,7 +18098,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-19 06:40</t>
+          <t>- 生成时间：2026-08-19 06:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31-F1-E-7-1 T-024 炮台默认值抽表数据侧(#3): GameData.xlsx +turret_config sheet 1行(id/damage/fire_interval/attack_range双行表头 se_auto_turret 5.0/0.5/220.0) + data_schema注册(dict形id主键 追加skill_icon_map后) + excel_export presentation段追加解析(数值coerce float) + files dict第6键 其余16JSON零diff
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -43,7 +43,8 @@
     <sheet name="spawn_points" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="boss_phase_events" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="skill_icon_map" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="总览" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="turret_config" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="总览" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$38</definedName>
@@ -18075,6 +18076,80 @@
 <file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fire_interval</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>attack_range</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>炮台ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>单发伤害</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>开火间隔(秒=cooldown)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>射程</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>se_auto_turret</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>220</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -18098,7 +18173,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-19 06:43</t>
+          <t>- 生成时间：2026-08-19 08:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day31-F1-E-5-1 T-020 icon_config抽表数据侧(#3): GameData.xlsx +icon_config sheet 3行(id/path/frame_count/frame_size_w/frame_size_h双行表头 weapons 40/items 54/skills 5 path与const现值一致 frame_size 32x32) + data_schema注册(dict形id主键 追加turret_config后) + excel_export presentation段追加解析(frame_size拆列组装) + files dict第7键 其余15JSON零diff + --check-only EXIT=0
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -44,7 +44,8 @@
     <sheet name="boss_phase_events" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="skill_icon_map" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="turret_config" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="总览" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="icon_config" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="总览" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'weapons'!$A$1:$AG$38</definedName>
@@ -18150,232 +18151,127 @@
 <file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t># 数据分布总览（DATA_OVERVIEW）</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>frame_count</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>frame_size_w</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>frame_size_h</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>图标集ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>资源路径</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>帧数</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>尺寸宽</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>尺寸高</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-19 08:45</t>
-        </is>
+          <t>weapons</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/ui/weapons.png</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>40</v>
+      </c>
+      <c r="D3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E3" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>- 来源：docs/GameData.xlsx（tools/excel_export.py 导出时自动刷新）</t>
-        </is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/ui/items.png</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>54</v>
+      </c>
+      <c r="D4" t="n">
+        <v>32</v>
+      </c>
+      <c r="E4" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>## weapons（37 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>- 分类分布：{'melee': 9, 'ranged': 10, 'elemental': 10, 'engineering': 8}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>- 等级条目：288（36 把 × 8 级）</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>- 基础 damage：min 0.0 / max 45.0 / 均值 11.8</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>- 基础 cooldown：min 0.05 / max 2.0 / 均值 0.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>- 基础 range：min 100.0 / max 400.0 / 均值 213.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>## items（54 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>- 稀有度分布：{'common': 15, 'uncommon': 12, 'rare': 12, 'legendary': 13, 'epic': 2}</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>- 效果键 Top（共 36 种）：damage_percent×14, max_hp×8, attack_speed_percent×7, armor×7, speed_percent×7, dodge_percent×6, elemental_damage×6, melee_damage×6</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>- price：min 0.0 / max 120.0 / 均值 57.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>## enemies（23 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>- 分类分布：{'regular': 15, 'elite': 6, 'boss': 2}</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>## characters（10 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>- 起始武器 10 把：pistol, fist, slingshot, wand, turret, dagger, se_star_flame, se_auto_turret, se_star_blade, se_holy_staff</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>## waves（20 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>- 波次范围：1 – 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>## events（10 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>## stats（20 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>## elements（6 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>## element_reactions（10 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>## routes（1 行）</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>## 关注项</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>- 无消费方效果键 17 个（T-050 已裁决：保留待 F2+/删数据）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, burn_duration_percent, damage_reduction_on_hit_percent, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, miss_chance_percent, no_weapon_armor_bonus, range, reaction_heal, special_enemies_next_wave, structure_duration_percent</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>skills</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>res://assets/sprites/skills/skills.png</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>32</v>
+      </c>
+      <c r="E5" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -20569,6 +20465,242 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:V56"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00808080"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t># 数据分布总览（DATA_OVERVIEW）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>- 生成时间：2026-08-19 12:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>- 来源：docs/GameData.xlsx（tools/excel_export.py 导出时自动刷新）</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>## weapons（37 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>- 分类分布：{'melee': 9, 'ranged': 10, 'elemental': 10, 'engineering': 8}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>- 等级条目：288（36 把 × 8 级）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>- 基础 damage：min 0.0 / max 45.0 / 均值 11.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>- 基础 cooldown：min 0.05 / max 2.0 / 均值 0.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>- 基础 range：min 100.0 / max 400.0 / 均值 213.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>## items（54 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- 稀有度分布：{'common': 15, 'uncommon': 12, 'rare': 12, 'legendary': 13, 'epic': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- 效果键 Top（共 36 种）：damage_percent×14, max_hp×8, attack_speed_percent×7, armor×7, speed_percent×7, dodge_percent×6, elemental_damage×6, melee_damage×6</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>- price：min 0.0 / max 120.0 / 均值 57.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>## enemies（23 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>- 分类分布：{'regular': 15, 'elite': 6, 'boss': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>## characters（10 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>- 起始武器 10 把：pistol, fist, slingshot, wand, turret, dagger, se_star_flame, se_auto_turret, se_star_blade, se_holy_staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>## waves（20 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>- 波次范围：1 – 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>## events（10 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>## stats（20 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>## elements（6 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>## element_reactions（10 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>## routes（1 行）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>## 关注项</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>- 无消费方效果键 17 个（T-050 已裁决：保留待 F2+/删数据）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, burn_duration_percent, damage_reduction_on_hit_percent, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, miss_chance_percent, no_weapon_armor_bonus, range, reaction_heal, special_enemies_next_wave, structure_duration_percent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Day31-RELIC-0-1 数据侧(#3): items relic 类条目 +6 新列(tag/tier/set_id/set_tier/set_effects/unlock_condition) + 套装2套4件占位(星骸孤注/死线舞者 price=0不进商店池) + 移速流派示例6件(T1×3/T2×2/T3×1) + items_effects子表+9行 + excel_export set_effects分隔串→JSON数组解析(方案定案 档:键=值;|) + KNOWN_EFFECT_KEYS+6新键 其余16JSON零diff
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -18281,7 +18281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V56"/>
+  <dimension ref="A1:AB66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="5"/>
@@ -18414,6 +18414,36 @@
           <t>trigger.speed_mult</t>
         </is>
       </c>
+      <c r="W1" s="6" t="inlineStr">
+        <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="X1" s="6" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="Y1" s="6" t="inlineStr">
+        <is>
+          <t>set_id</t>
+        </is>
+      </c>
+      <c r="Z1" s="6" t="inlineStr">
+        <is>
+          <t>set_tier</t>
+        </is>
+      </c>
+      <c r="AA1" s="6" t="inlineStr">
+        <is>
+          <t>set_effects</t>
+        </is>
+      </c>
+      <c r="AB1" s="6" t="inlineStr">
+        <is>
+          <t>unlock_condition</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18526,6 +18556,36 @@
           <t>触发.速度倍率</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>流派标签</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>档位</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>套装ID</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>套装档位</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>套装效果(档:键=值;分隔)</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>解锁条件</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -20269,6 +20329,14 @@
       <c r="I52" t="n">
         <v>49</v>
       </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="X52" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -20302,6 +20370,14 @@
       <c r="I53" t="n">
         <v>50</v>
       </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>engineering</t>
+        </is>
+      </c>
+      <c r="X53" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -20457,6 +20533,503 @@
       </c>
       <c r="V56" t="n">
         <v>1.2</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>relic_starbound_heart</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>星骸之心</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>["relic","offense"]</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>49</v>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>offense</t>
+        </is>
+      </c>
+      <c r="X57" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>starbound_gamble</t>
+        </is>
+      </c>
+      <c r="Z57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>1:max_hp_percent=-90;damage_taken_percent=-40|2:damage_percent=100;attack_speed_percent=50;damage_taken_percent=-30</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr">
+        <is>
+          <t>first_kill_boss:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>relic_starbound_core</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>星骸核心</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>["relic","offense"]</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>50</v>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>offense</t>
+        </is>
+      </c>
+      <c r="X58" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>starbound_gamble</t>
+        </is>
+      </c>
+      <c r="Z58" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>1:max_hp_percent=-90;damage_taken_percent=-40|2:damage_percent=100;attack_speed_percent=50;damage_taken_percent=-30</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr">
+        <is>
+          <t>first_kill_boss:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>relic_deadline_boots</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>死线舞靴</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>49</v>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X59" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>deadline_dancer</t>
+        </is>
+      </c>
+      <c r="Z59" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>1:max_hp_percent=-70;speed_percent=30|2:move_stacking_damage=1</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>first_kill_boss:2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>relic_deadline_heels</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>死线舞跟</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>50</v>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X60" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y60" t="inlineStr">
+        <is>
+          <t>deadline_dancer</t>
+        </is>
+      </c>
+      <c r="Z60" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA60" t="inlineStr">
+        <is>
+          <t>1:max_hp_percent=-70;speed_percent=30|2:move_stacking_damage=1</t>
+        </is>
+      </c>
+      <c r="AB60" t="inlineStr">
+        <is>
+          <t>first_kill_boss:2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>relic_swift_feet</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>疾行靴</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>49</v>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>relic_swift_trade</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>轻装契约</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>49</v>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>relic_swift_dodge</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>残影步</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>49</v>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>relic_swift_kinetic</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>动能转化</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>0</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>49</v>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X64" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB64" t="inlineStr">
+        <is>
+          <t>fail_count&gt;=3</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>relic_swift_rush</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>冲刺余波</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>49</v>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X65" t="n">
+        <v>2</v>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t>codex_count&gt;=10</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>relic_swift_split</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>音速分裂</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>["relic","speed"]</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>relic</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>49</v>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="X66" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB66" t="inlineStr">
+        <is>
+          <t>affinity_tag&gt;=3</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -20491,7 +21064,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-19 18:39</t>
+          <t>- 生成时间：2026-08-19 20:44</t>
         </is>
       </c>
     </row>
@@ -20553,28 +21126,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>## items（54 行）</t>
+          <t>## items（64 行）</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>- 稀有度分布：{'common': 15, 'uncommon': 12, 'rare': 12, 'legendary': 13, 'epic': 2}</t>
+          <t>- 稀有度分布：{'common': 18, 'uncommon': 14, 'rare': 17, 'legendary': 13, 'epic': 2}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>- 效果键 Top（共 36 种）：damage_percent×14, max_hp×8, attack_speed_percent×7, armor×7, speed_percent×7, dodge_percent×6, elemental_damage×6, melee_damage×6</t>
+          <t>- 效果键 Top（共 40 种）：damage_percent×14, speed_percent×10, armor×8, max_hp×8, attack_speed_percent×7, dodge_percent×7, elemental_damage×6, melee_damage×6</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- price：min 0.0 / max 120.0 / 均值 57.2</t>
+          <t>- price：min 0.0 / max 120.0 / 均值 48.3</t>
         </is>
       </c>
     </row>
@@ -20692,7 +21265,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>- 无消费方效果键 17 个（T-050 已裁决：保留待 F2+/删数据）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, burn_duration_percent, damage_reduction_on_hit_percent, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, miss_chance_percent, no_weapon_armor_bonus, range, reaction_heal, special_enemies_next_wave, structure_duration_percent</t>
+          <t>- 无消费方效果键 23 个（T-050 已裁决：保留待 F2+/删数据）：attack_speed_per_different_weapon_percent, auto_turret_per_wave, burn_duration_percent, damage_reduction_on_hit_percent, distance_trigger, dodge_heal_amount, dodge_heal_chance, element_duration_percent, element_reaction_damage_percent, engineering, fire_damage_percent, harvesting, max_hp_percent, miss_chance_percent, move_speed_threshold, move_speed_to_damage_percent, move_stacking_damage, no_weapon_armor_bonus, projectile_split, range, reaction_heal, special_enemies_next_wave, structure_duration_percent</t>
         </is>
       </c>
     </row>
@@ -20707,7 +21280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C131"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -22546,6 +23119,141 @@
       </c>
       <c r="C122" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>relic_swift_feet</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>speed_percent</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>relic_swift_trade</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>speed_percent</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>relic_swift_trade</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>relic_swift_dodge</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>speed_percent</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>relic_swift_dodge</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>dodge_percent</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>relic_swift_kinetic</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>move_speed_to_damage_percent</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>relic_swift_rush</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>distance_trigger</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>relic_swift_split</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>move_speed_threshold</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>relic_swift_split</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>projectile_split</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day31-RELIC-F1 数据侧(#3): boss_pattern表+3节奏列(cast_slowdown施放站定0.0/chase_ratio追踪系数0.2/skill_window走位1.0s, circle系3行) 导出boss_patterns.json带新键 其余16JSON零diff
</commit_message>
<xml_diff>
--- a/docs/GameData.xlsx
+++ b/docs/GameData.xlsx
@@ -8841,7 +8841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="4"/>
   <sheetData>
     <row r="1">
@@ -8875,6 +8875,21 @@
           <t>min_interval</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>cast_slowdown</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>chase_ratio</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>skill_window</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8907,6 +8922,21 @@
           <t>最短释放间隔(s)</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>施放期移速倍率(0=站定)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>追踪段时长系数(冷却x系数)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>施放后走位时长(s)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8933,6 +8963,15 @@
       <c r="F3" t="n">
         <v>4</v>
       </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8959,6 +8998,15 @@
       <c r="F4" t="n">
         <v>6</v>
       </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8984,6 +9032,15 @@
       </c>
       <c r="F5" t="n">
         <v>4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -21064,7 +21121,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>- 生成时间：2026-08-19 20:44</t>
+          <t>- 生成时间：2026-08-19 22:40</t>
         </is>
       </c>
     </row>

</xml_diff>